<commit_message>
Revert "Add files via upload"
This reverts commit bc586a7391c8dc4e9f5c6565fb516b138cc19b7f.
</commit_message>
<xml_diff>
--- a/atom01_pcb/Roboto_Usb2Can/02_Assembly/HUB-USB2CAN_Bom.xlsx
+++ b/atom01_pcb/Roboto_Usb2Can/02_Assembly/HUB-USB2CAN_Bom.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Roboto_Usb2Can_V1.0_1_Robot" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_PCB1_2026-01-08" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="152">
   <si>
     <t>No.</t>
   </si>
@@ -37,37 +37,37 @@
     <t>1</t>
   </si>
   <si>
+    <t>100nF</t>
+  </si>
+  <si>
+    <t>C2,C3,C4,C5,C6,C7,C8,C14,C15,C16,C17,C18,C19,C20,C21,C22,C23,C24,C28,C29,C30,C31,C32,C33,C34,C35,C36,C37,C38,C44,C46,C47,C48,C49,C50,C51,C52,C58,C76,C77,C78,C79</t>
+  </si>
+  <si>
+    <t>C0402</t>
+  </si>
+  <si>
+    <t>CL05B104KB54PNC</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>1uF</t>
   </si>
   <si>
-    <t>C1,C5</t>
-  </si>
-  <si>
-    <t>C0402</t>
+    <t>C9,C10</t>
   </si>
   <si>
     <t>CL05A105KA5NQNC</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>100nF</t>
-  </si>
-  <si>
-    <t>C2,C3,C4,C6,C7,C8,C9,C10,C11,C12,C13,C14,C19,C20,C21,C22,C23,C24,C26,C27,C28,C31,C32,C33,C34,C35,C36,C37,C38,C39,C40,C41,C42,C43,C44,C45,C46,C47,C48,C49,C50,C51</t>
-  </si>
-  <si>
-    <t>CL05B104KB54PNC</t>
-  </si>
-  <si>
     <t>3</t>
   </si>
   <si>
     <t>10uF</t>
   </si>
   <si>
-    <t>C15,C16</t>
+    <t>C61,C62,C71,C72</t>
   </si>
   <si>
     <t>C0603</t>
@@ -79,7 +79,7 @@
     <t>4</t>
   </si>
   <si>
-    <t>C17,C18</t>
+    <t>C63,C64</t>
   </si>
   <si>
     <t>06035C104JAT2A</t>
@@ -91,7 +91,7 @@
     <t>12pF</t>
   </si>
   <si>
-    <t>C25,C30</t>
+    <t>C73,C74</t>
   </si>
   <si>
     <t>CC0603JRNPO9BN120</t>
@@ -103,7 +103,7 @@
     <t>22uF</t>
   </si>
   <si>
-    <t>C29</t>
+    <t>C75</t>
   </si>
   <si>
     <t>CGA0603X5R226M160JT</t>
@@ -115,10 +115,10 @@
     <t>0Ω</t>
   </si>
   <si>
-    <t>CS1,CS2,CS3,CS4,R6</t>
-  </si>
-  <si>
-    <t>R0603_1</t>
+    <t>CS1,CS2,CS3,CS4,R75</t>
+  </si>
+  <si>
+    <t>R0603</t>
   </si>
   <si>
     <t>0603WAF0000T5E</t>
@@ -130,7 +130,7 @@
     <t>ESDA6V1L</t>
   </si>
   <si>
-    <t>D1,D2,D3,D4</t>
+    <t>D2,D3,D4,D5</t>
   </si>
   <si>
     <t>SOT-23-3_L2.9-W1.3-P1.90-LS2.4-BR</t>
@@ -148,7 +148,7 @@
     <t>SMBJ6.0CA</t>
   </si>
   <si>
-    <t>D5</t>
+    <t>D6</t>
   </si>
   <si>
     <t>SMB_L4.6-W3.6-LS5.3-BI</t>
@@ -172,39 +172,39 @@
     <t>11</t>
   </si>
   <si>
+    <t>SZYY0603B</t>
+  </si>
+  <si>
+    <t>LED1,LED6,LED7,LED9,LED10,LED12,LED13,LED15</t>
+  </si>
+  <si>
+    <t>LED0603-R-RD_BLUE</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>SZYY0603G</t>
+  </si>
+  <si>
+    <t>LED3,LED8,LED11,LED14</t>
+  </si>
+  <si>
+    <t>LED0603-R-RD_GREEN</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
     <t>NCD0603Y2</t>
   </si>
   <si>
-    <t>LED1</t>
+    <t>LED16</t>
   </si>
   <si>
     <t>LED0603-RD</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>SZYY0603B</t>
-  </si>
-  <si>
-    <t>LED2,LED3,LED5,LED6,LED8,LED9,LED11,LED12</t>
-  </si>
-  <si>
-    <t>LED0603-R-RD_BLUE</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>SZYY0603G</t>
-  </si>
-  <si>
-    <t>LED4,LED7,LED10,LED13</t>
-  </si>
-  <si>
-    <t>LED0603-R-RD_GREEN</t>
-  </si>
-  <si>
     <t>14</t>
   </si>
   <si>
@@ -232,25 +232,34 @@
     <t>16</t>
   </si>
   <si>
+    <t>2kΩ</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>0603WAF2001T5E</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
     <t>5.1kΩ</t>
   </si>
   <si>
-    <t>R1,R3</t>
-  </si>
-  <si>
-    <t>R0603</t>
+    <t>R2,R3</t>
   </si>
   <si>
     <t>TNPW06035K10BEEA</t>
   </si>
   <si>
-    <t>17</t>
+    <t>18</t>
   </si>
   <si>
     <t>10kΩ</t>
   </si>
   <si>
-    <t>R2,R7,R25,R26,R27,R28,R29,R30</t>
+    <t>R5,R63,R79,R80,R90,R91,R101,R102</t>
   </si>
   <si>
     <t>R0402</t>
@@ -259,73 +268,61 @@
     <t>0402WGF1002TCE</t>
   </si>
   <si>
-    <t>18</t>
+    <t>19</t>
+  </si>
+  <si>
+    <t>1MΩ</t>
+  </si>
+  <si>
+    <t>R8</t>
+  </si>
+  <si>
+    <t>0603WAF1004T5E</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>100kΩ</t>
+  </si>
+  <si>
+    <t>R9</t>
+  </si>
+  <si>
+    <t>RCA03100KJLF</t>
+  </si>
+  <si>
+    <t>21</t>
   </si>
   <si>
     <t>120Ω</t>
   </si>
   <si>
-    <t>R4,R5,R9,R10</t>
+    <t>R74,R85,R96,R107</t>
   </si>
   <si>
     <t>0603WAF1200T5E</t>
   </si>
   <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>2kΩ</t>
-  </si>
-  <si>
-    <t>R8</t>
-  </si>
-  <si>
-    <t>0603WAF2001T5E</t>
-  </si>
-  <si>
-    <t>20</t>
+    <t>22</t>
   </si>
   <si>
     <t>1kΩ</t>
   </si>
   <si>
-    <t>R11,R12,R13,R14,R15,R16,R17,R18,R21,R22,R23,R24</t>
+    <t>R76,R77,R78,R87,R88,R89,R98,R99,R100,R109,R110,R111</t>
   </si>
   <si>
     <t>0603WAF1001T5E</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>1MΩ</t>
-  </si>
-  <si>
-    <t>R19</t>
-  </si>
-  <si>
-    <t>0603WAF1004T5E</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>100kΩ</t>
-  </si>
-  <si>
-    <t>R20</t>
-  </si>
-  <si>
-    <t>RCA03100KJLF</t>
-  </si>
-  <si>
     <t>23</t>
   </si>
   <si>
     <t>VPT85BB-01A</t>
   </si>
   <si>
-    <t>T1,T2</t>
+    <t>T3,T4</t>
   </si>
   <si>
     <t>XFMR-SMD_L7.5-W6.7-P2.54-LS7.7-BL</t>
@@ -346,109 +343,109 @@
     <t>25</t>
   </si>
   <si>
+    <t>STM32G431C8T6</t>
+  </si>
+  <si>
+    <t>U1,U26,U34,U42</t>
+  </si>
+  <si>
+    <t>LQFP-48_L7.0-W7.0-P0.50-LS9.0-BL</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>VPS8505</t>
+  </si>
+  <si>
+    <t>U20,U29</t>
+  </si>
+  <si>
+    <t>SOT-23-6_L2.9-W1.6-P0.95-LS2.8-BR</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>DSK36</t>
+  </si>
+  <si>
+    <t>U21,U22,U30,U31</t>
+  </si>
+  <si>
+    <t>SOD-123FL_L2.8-W1.9-LS3.7-RD</t>
+  </si>
+  <si>
+    <t>DSK36_C22466353</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>TPS76350DBVR-TP</t>
+  </si>
+  <si>
+    <t>U24,U32</t>
+  </si>
+  <si>
+    <t>SOT-23-5_L3.0-W1.6-P0.95-LS2.8-BR</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>ISO1050DWR</t>
+  </si>
+  <si>
+    <t>U25,U33,U41,U49</t>
+  </si>
+  <si>
+    <t>SOIC-16_L10.3-W7.5-P1.27-LS10.3-BL</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>SL2.1A</t>
+  </si>
+  <si>
+    <t>U50</t>
+  </si>
+  <si>
+    <t>SOP-16_L10.0-W3.9-P1.27-LS6.0-BL</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>SM02B-GHS-TB(LF)(SN)</t>
+  </si>
+  <si>
+    <t>U52,U53,U54,U55</t>
+  </si>
+  <si>
+    <t>CONN-SMD_SM02B-GHS-TB-LF-SN</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
     <t>TLV75733PDBVR</t>
   </si>
   <si>
-    <t>U1</t>
+    <t>U56</t>
   </si>
   <si>
     <t>SOT-23-5_L2.9-W1.6-P0.95-LS2.8-BL</t>
   </si>
   <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>ISO1050DWR</t>
-  </si>
-  <si>
-    <t>U2,U3,U5,U6</t>
-  </si>
-  <si>
-    <t>SOIC-16_L10.3-W7.5-P1.27-LS10.3-BL</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>STM32G431C8T6</t>
-  </si>
-  <si>
-    <t>U4,U16,U17,U18</t>
-  </si>
-  <si>
-    <t>LQFP-48_L7.0-W7.0-P0.50-LS9.0-BL</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>DSK36</t>
-  </si>
-  <si>
-    <t>U7,U11,U12,U15</t>
-  </si>
-  <si>
-    <t>SOD-123FL_L2.8-W1.9-LS3.7-RD</t>
-  </si>
-  <si>
-    <t>DSK36_C22466353</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>TPS76350DBVR-TP</t>
-  </si>
-  <si>
-    <t>U8,U13</t>
-  </si>
-  <si>
-    <t>SOT-23-5_L3.0-W1.6-P0.95-LS2.8-BR</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>VPS8505</t>
-  </si>
-  <si>
-    <t>U9,U14</t>
-  </si>
-  <si>
-    <t>SOT-23-6_L2.9-W1.6-P0.95-LS2.8-BR</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>SL2.1A</t>
-  </si>
-  <si>
-    <t>U10</t>
-  </si>
-  <si>
-    <t>SOP-16_L10.0-W3.9-P1.27-LS6.0-BL</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>SM02B-GHS-TB(LF)(SN)</t>
-  </si>
-  <si>
-    <t>U19,U20,U21,U22</t>
-  </si>
-  <si>
-    <t>CONN-SMD_SM02B-GHS-TB-LF-SN</t>
-  </si>
-  <si>
     <t>33</t>
   </si>
   <si>
     <t>TYPEC-304-BCP16</t>
   </si>
   <si>
-    <t>USB1</t>
+    <t>USB9</t>
   </si>
   <si>
     <t>USB-C-SMD_TYPEC-304-BCP16</t>
@@ -463,7 +460,7 @@
     <t>12MHz</t>
   </si>
   <si>
-    <t>X1</t>
+    <t>X2</t>
   </si>
   <si>
     <t>CRYSTAL-SMD_4P-L3.2-W2.5-BL</t>
@@ -880,7 +877,7 @@
         <v>7</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -903,7 +900,7 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -926,7 +923,7 @@
         <v>16</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
@@ -952,7 +949,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
         <v>22</v>
@@ -961,7 +958,7 @@
         <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G5" t="s">
         <v>23</v>
@@ -1110,7 +1107,7 @@
         <v>52</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C12" t="s">
         <v>53</v>
@@ -1133,7 +1130,7 @@
         <v>56</v>
       </c>
       <c r="B13">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C13" t="s">
         <v>57</v>
@@ -1156,7 +1153,7 @@
         <v>60</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C14" t="s">
         <v>61</v>
@@ -1225,7 +1222,7 @@
         <v>72</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" t="s">
         <v>73</v>
@@ -1234,266 +1231,266 @@
         <v>74</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="F17" t="s">
         <v>73</v>
       </c>
       <c r="G17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
         <v>77</v>
       </c>
-      <c r="B18">
-        <v>8</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>78</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" t="s">
         <v>79</v>
-      </c>
-      <c r="E18" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" t="s">
-        <v>78</v>
-      </c>
-      <c r="G18" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" t="s">
         <v>82</v>
       </c>
-      <c r="B19">
-        <v>4</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
         <v>83</v>
       </c>
-      <c r="D19" t="s">
+      <c r="F19" t="s">
+        <v>81</v>
+      </c>
+      <c r="G19" t="s">
         <v>84</v>
-      </c>
-      <c r="E19" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" t="s">
-        <v>83</v>
-      </c>
-      <c r="G19" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" t="s">
         <v>87</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20" t="s">
+        <v>86</v>
+      </c>
+      <c r="G20" t="s">
         <v>88</v>
-      </c>
-      <c r="E20" t="s">
-        <v>75</v>
-      </c>
-      <c r="F20" t="s">
-        <v>87</v>
-      </c>
-      <c r="G20" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
         <v>90</v>
       </c>
-      <c r="B21">
-        <v>12</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>91</v>
-      </c>
-      <c r="D21" t="s">
-        <v>92</v>
       </c>
       <c r="E21" t="s">
         <v>35</v>
       </c>
       <c r="F21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B22">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
         <v>94</v>
       </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>95</v>
-      </c>
-      <c r="D22" t="s">
-        <v>96</v>
       </c>
       <c r="E22" t="s">
         <v>35</v>
       </c>
       <c r="F22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
         <v>98</v>
       </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>99</v>
-      </c>
-      <c r="D23" t="s">
-        <v>100</v>
       </c>
       <c r="E23" t="s">
         <v>35</v>
       </c>
       <c r="F23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B24">
         <v>2</v>
       </c>
       <c r="C24" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" t="s">
         <v>103</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>104</v>
       </c>
-      <c r="E24" t="s">
-        <v>105</v>
-      </c>
       <c r="F24" t="s">
         <v>41</v>
       </c>
       <c r="G24" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B25">
         <v>16</v>
       </c>
       <c r="C25" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" t="s">
         <v>107</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>108</v>
       </c>
-      <c r="E25" t="s">
-        <v>109</v>
-      </c>
       <c r="F25" t="s">
         <v>41</v>
       </c>
       <c r="G25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
         <v>110</v>
       </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>111</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>112</v>
       </c>
-      <c r="E26" t="s">
-        <v>113</v>
-      </c>
       <c r="F26" t="s">
         <v>41</v>
       </c>
       <c r="G26" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27">
+        <v>2</v>
+      </c>
+      <c r="C27" t="s">
         <v>114</v>
       </c>
-      <c r="B27">
-        <v>4</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>115</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>116</v>
       </c>
-      <c r="E27" t="s">
-        <v>117</v>
-      </c>
       <c r="F27" t="s">
         <v>41</v>
       </c>
       <c r="G27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B28">
         <v>4</v>
       </c>
       <c r="C28" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" t="s">
         <v>119</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>120</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
+        <v>41</v>
+      </c>
+      <c r="G28" t="s">
         <v>121</v>
-      </c>
-      <c r="F28" t="s">
-        <v>41</v>
-      </c>
-      <c r="G28" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1501,7 +1498,7 @@
         <v>122</v>
       </c>
       <c r="B29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C29" t="s">
         <v>123</v>
@@ -1516,145 +1513,145 @@
         <v>41</v>
       </c>
       <c r="G29" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30">
+        <v>4</v>
+      </c>
+      <c r="C30" t="s">
         <v>127</v>
       </c>
-      <c r="B30">
-        <v>2</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>128</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>129</v>
       </c>
-      <c r="E30" t="s">
-        <v>130</v>
-      </c>
       <c r="F30" t="s">
         <v>41</v>
       </c>
       <c r="G30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
         <v>131</v>
       </c>
-      <c r="B31">
-        <v>2</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>132</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>133</v>
       </c>
-      <c r="E31" t="s">
-        <v>134</v>
-      </c>
       <c r="F31" t="s">
         <v>41</v>
       </c>
       <c r="G31" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>134</v>
+      </c>
+      <c r="B32">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
         <v>135</v>
       </c>
-      <c r="B32">
-        <v>1</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>136</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>137</v>
       </c>
-      <c r="E32" t="s">
-        <v>138</v>
-      </c>
       <c r="F32" t="s">
         <v>41</v>
       </c>
       <c r="G32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>138</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
         <v>139</v>
       </c>
-      <c r="B33">
-        <v>4</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>140</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>141</v>
       </c>
-      <c r="E33" t="s">
-        <v>142</v>
-      </c>
       <c r="F33" t="s">
         <v>41</v>
       </c>
       <c r="G33" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B34">
         <v>1</v>
       </c>
       <c r="C34" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" t="s">
         <v>144</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>145</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
+        <v>41</v>
+      </c>
+      <c r="G34" t="s">
         <v>146</v>
-      </c>
-      <c r="F34" t="s">
-        <v>41</v>
-      </c>
-      <c r="G34" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B35">
         <v>1</v>
       </c>
       <c r="C35" t="s">
+        <v>148</v>
+      </c>
+      <c r="D35" t="s">
         <v>149</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>150</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
+        <v>148</v>
+      </c>
+      <c r="G35" t="s">
         <v>151</v>
-      </c>
-      <c r="F35" t="s">
-        <v>149</v>
-      </c>
-      <c r="G35" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>